<commit_message>
chore: publish xdsdocuments IG 0.1.0-homecareobservation-draft-2
</commit_message>
<xml_diff>
--- a/ig/xdsdocuments/CodeSystem-MedComHCOFormatCodeCS.xlsx
+++ b/ig/xdsdocuments/CodeSystem-MedComHCOFormatCodeCS.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0-homecareobservation-draft</t>
+    <t>0.1.0-homecareobservation-draft-2</t>
   </si>
   <si>
     <t>Name</t>
@@ -45,7 +45,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-16T11:19:10+00:00</t>
+    <t>2026-04-30T11:35:54+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
chore: publish xdsdocuments IG 0.1.0-homecareobservation-draft-2 (#77)
Co-authored-by: olw-medcom <olw-medcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/xdsdocuments/CodeSystem-MedComHCOFormatCodeCS.xlsx
+++ b/ig/xdsdocuments/CodeSystem-MedComHCOFormatCodeCS.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0-homecareobservation-draft</t>
+    <t>0.1.0-homecareobservation-draft-2</t>
   </si>
   <si>
     <t>Name</t>
@@ -45,7 +45,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-16T11:19:10+00:00</t>
+    <t>2026-04-30T11:35:54+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>